<commit_message>
update log, fixe calendar dates
</commit_message>
<xml_diff>
--- a/Content_Calendar.xlsx
+++ b/Content_Calendar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John\Desktop\content calendar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8679989-700A-402E-B4AA-6246D78F7734}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7891210E-2699-4F0C-9E88-6150910EBABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="51840" windowHeight="21840" xr2:uid="{FA463503-EEA9-4E36-AF77-605EC82561F6}"/>
   </bookViews>
@@ -335,9 +335,6 @@
     <t>This is Chita. She is 8 years old and lives in Cambodia. \n\n📸 We gave her a camera and asked her to take a picture of what she finds beautiful in the world. Chita decided to take a picture of the “kontout” fruit tree.\n\nShe said, “I photographed this tree because the fruit tastes very good. Sweet and sour. I like them.”\n\nLet’s not forget the beauty that surrounds us everyday. Let’s see the world like Chita does.</t>
   </si>
   <si>
-    <t>When you think of the perfect Christmas gift, you may not think of chickens.\n\nBut you might when you hear Betty and Michal’s inspiring story.\n\n“Now we can be sure to eat two meals a day. We have enough money to buy food. My children are healthy,” Betty says. 🙏 \n\nIsn’t that beautiful? \n\nBefore someone caring made room for gifts of love, their family struggled with hunger and uncertainty. Everything changed when someone like you sent chickens and seeds that helped them grow food, earn income and dream again.\n\nYou can help another family put food on the table now and for years to come.\n\nShop the Gift Catalog online &gt; www.fh.org/shop</t>
-  </si>
-  <si>
     <t>“My children were malnourished and we hardly ate one meal a day,” says Betty in Uganda. \n\nBetty and Michal struggled to feed their daughters and pay school fees. But everything changed when kind people like you helped change their lives with gifts from the Food for the Hungry Gift Catalog. \n \n Chickens to lay eggs. Seeds to grow vegetables. Tools and training to build a future. \n \n “Now we eat two meals a day. My children are healthy. We have hope,” Betty shares. 🫶 \n\nThis Christmas, you can give a gift that puts food on the table and changes lives.</t>
   </si>
   <si>
@@ -548,6 +545,9 @@
   </si>
   <si>
     <t>Grateful for the incredible community and church leaders coming together as Church of the City in Franklin, Tennessee has been building powerful partnership with the community of La Cuneta in the Dominican Republic. \n\n  Excited for the journey ahead as we work hand in hand to bring hope, love, and lasting impact!</t>
+  </si>
+  <si>
+    <t>When you think of the perfect Christmas gift, you may not think of chickens.\n\nBut you might when you hear Betty and Michal’s inspiring story.\n\n“Now we can be sure to eat two meals a day. We have enough money to buy food. My children are healthy,” Betty says. 🙏 \n\nIsn’t that beautiful? \n\nBefore someone caring made room for gifts of love, their family struggled with hunger and uncertainty. Everything changed when someone like you sent chickens and seeds that helped them grow food, earn income and dream again.\n\nYou can help another family put food on the table now and for years to come.</t>
   </si>
 </sst>
 </file>
@@ -1066,7 +1066,7 @@
         <v>21</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H2" s="4" t="s">
         <v>22</v>
@@ -1105,7 +1105,7 @@
         <v>26</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>20</v>
@@ -1114,7 +1114,7 @@
         <v>27</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H3" s="4" t="s">
         <v>22</v>
@@ -1159,10 +1159,10 @@
         <v>20</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>107</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>22</v>
@@ -1189,7 +1189,7 @@
         <v>23</v>
       </c>
       <c r="R4" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" spans="1:18" ht="105" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>33</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>22</v>
@@ -1402,7 +1402,7 @@
         <v>43</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>22</v>
@@ -1573,10 +1573,10 @@
         <v>23</v>
       </c>
       <c r="R12" s="8" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" ht="120" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="60" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>17</v>
       </c>
@@ -1585,7 +1585,7 @@
         <v>26</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>20</v>
@@ -1594,7 +1594,7 @@
         <v>53</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>99</v>
+        <v>167</v>
       </c>
       <c r="H13" s="4" t="s">
         <v>22</v>
@@ -1681,7 +1681,7 @@
         <v>26</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>20</v>
@@ -1731,10 +1731,10 @@
         <v>20</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H16" s="4" t="s">
         <v>22</v>
@@ -1779,10 +1779,10 @@
         <v>20</v>
       </c>
       <c r="F17" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="G17" s="2" t="s">
         <v>110</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>111</v>
       </c>
       <c r="H17" s="4" t="s">
         <v>22</v>
@@ -1809,7 +1809,7 @@
         <v>23</v>
       </c>
       <c r="R17" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.25">
@@ -1869,7 +1869,7 @@
         <v>26</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>20</v>
@@ -1878,7 +1878,7 @@
         <v>68</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H19" s="4" t="s">
         <v>22</v>
@@ -1917,16 +1917,16 @@
         <v>26</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H20" s="4" t="s">
         <v>22</v>
@@ -1974,7 +1974,7 @@
         <v>70</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H21" s="4" t="s">
         <v>22</v>
@@ -2001,7 +2001,7 @@
         <v>23</v>
       </c>
       <c r="R21" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="22" spans="1:18" ht="135" x14ac:dyDescent="0.25">
@@ -2022,7 +2022,7 @@
         <v>72</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H22" s="4" t="s">
         <v>22</v>
@@ -2037,10 +2037,10 @@
         <v>23</v>
       </c>
       <c r="N22" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="O22" s="3" t="s">
         <v>126</v>
-      </c>
-      <c r="O22" s="3" t="s">
-        <v>127</v>
       </c>
       <c r="P22" s="3" t="s">
         <v>23</v>
@@ -2070,7 +2070,7 @@
         <v>21</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H23" s="4" t="s">
         <v>22</v>
@@ -2118,7 +2118,7 @@
         <v>31</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H24" s="4" t="s">
         <v>22</v>
@@ -2136,7 +2136,7 @@
         <v>57</v>
       </c>
       <c r="O24" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="P24" s="3" t="s">
         <v>23</v>
@@ -2163,10 +2163,10 @@
         <v>20</v>
       </c>
       <c r="F25" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="G25" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>107</v>
       </c>
       <c r="H25" s="4" t="s">
         <v>22</v>
@@ -2193,7 +2193,7 @@
         <v>23</v>
       </c>
       <c r="R25" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="26" spans="1:18" ht="45" x14ac:dyDescent="0.25">
@@ -2262,7 +2262,7 @@
         <v>84</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H27" s="4" t="s">
         <v>22</v>
@@ -2310,7 +2310,7 @@
         <v>33</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H28" s="4" t="s">
         <v>22</v>
@@ -2358,7 +2358,7 @@
         <v>43</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H29" s="4" t="s">
         <v>22</v>
@@ -2406,7 +2406,7 @@
         <v>53</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="H30" s="4" t="s">
         <v>22</v>
@@ -2492,16 +2492,16 @@
         <v>18</v>
       </c>
       <c r="D32" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E32" t="s">
         <v>20</v>
       </c>
       <c r="F32" t="s">
+        <v>132</v>
+      </c>
+      <c r="G32" t="s">
         <v>133</v>
-      </c>
-      <c r="G32" t="s">
-        <v>134</v>
       </c>
       <c r="H32" t="s">
         <v>22</v>
@@ -2525,7 +2525,7 @@
         <v>23</v>
       </c>
       <c r="R32" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.25">
@@ -2536,16 +2536,16 @@
         <v>26</v>
       </c>
       <c r="D33" t="s">
+        <v>135</v>
+      </c>
+      <c r="E33" t="s">
+        <v>20</v>
+      </c>
+      <c r="F33" t="s">
         <v>136</v>
       </c>
-      <c r="E33" t="s">
-        <v>20</v>
-      </c>
-      <c r="F33" t="s">
+      <c r="G33" t="s">
         <v>137</v>
-      </c>
-      <c r="G33" t="s">
-        <v>138</v>
       </c>
       <c r="H33" t="s">
         <v>22</v>
@@ -2569,7 +2569,7 @@
         <v>23</v>
       </c>
       <c r="R33" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.25">
@@ -2580,16 +2580,16 @@
         <v>26</v>
       </c>
       <c r="D34" t="s">
+        <v>139</v>
+      </c>
+      <c r="E34" t="s">
+        <v>20</v>
+      </c>
+      <c r="F34" t="s">
         <v>140</v>
       </c>
-      <c r="E34" t="s">
-        <v>20</v>
-      </c>
-      <c r="F34" t="s">
+      <c r="G34" t="s">
         <v>141</v>
-      </c>
-      <c r="G34" t="s">
-        <v>142</v>
       </c>
       <c r="H34" t="s">
         <v>22</v>
@@ -2613,7 +2613,7 @@
         <v>23</v>
       </c>
       <c r="R34" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.25">
@@ -2624,16 +2624,16 @@
         <v>26</v>
       </c>
       <c r="D35" t="s">
+        <v>143</v>
+      </c>
+      <c r="E35" t="s">
+        <v>20</v>
+      </c>
+      <c r="F35" t="s">
+        <v>162</v>
+      </c>
+      <c r="G35" t="s">
         <v>144</v>
-      </c>
-      <c r="E35" t="s">
-        <v>20</v>
-      </c>
-      <c r="F35" t="s">
-        <v>163</v>
-      </c>
-      <c r="G35" t="s">
-        <v>145</v>
       </c>
       <c r="H35" t="s">
         <v>22</v>
@@ -2657,7 +2657,7 @@
         <v>23</v>
       </c>
       <c r="R35" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.25">
@@ -2668,16 +2668,16 @@
         <v>26</v>
       </c>
       <c r="D36" t="s">
+        <v>146</v>
+      </c>
+      <c r="E36" t="s">
+        <v>20</v>
+      </c>
+      <c r="F36" t="s">
         <v>147</v>
       </c>
-      <c r="E36" t="s">
-        <v>20</v>
-      </c>
-      <c r="F36" t="s">
+      <c r="G36" t="s">
         <v>148</v>
-      </c>
-      <c r="G36" t="s">
-        <v>149</v>
       </c>
       <c r="H36" t="s">
         <v>22</v>
@@ -2701,7 +2701,7 @@
         <v>23</v>
       </c>
       <c r="R36" s="8" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.25">
@@ -2712,16 +2712,16 @@
         <v>26</v>
       </c>
       <c r="D37" t="s">
+        <v>150</v>
+      </c>
+      <c r="E37" t="s">
+        <v>20</v>
+      </c>
+      <c r="F37" t="s">
         <v>151</v>
       </c>
-      <c r="E37" t="s">
-        <v>20</v>
-      </c>
-      <c r="F37" t="s">
+      <c r="G37" t="s">
         <v>152</v>
-      </c>
-      <c r="G37" t="s">
-        <v>153</v>
       </c>
       <c r="H37" t="s">
         <v>22</v>
@@ -2745,7 +2745,7 @@
         <v>23</v>
       </c>
       <c r="R37" s="8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.25">
@@ -2756,16 +2756,16 @@
         <v>26</v>
       </c>
       <c r="D38" t="s">
+        <v>154</v>
+      </c>
+      <c r="E38" t="s">
+        <v>20</v>
+      </c>
+      <c r="F38" t="s">
         <v>155</v>
       </c>
-      <c r="E38" t="s">
-        <v>20</v>
-      </c>
-      <c r="F38" t="s">
+      <c r="G38" t="s">
         <v>156</v>
-      </c>
-      <c r="G38" t="s">
-        <v>157</v>
       </c>
       <c r="H38" t="s">
         <v>22</v>
@@ -2777,7 +2777,7 @@
         <v>22</v>
       </c>
       <c r="N38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="O38" t="s">
         <v>58</v>
@@ -2800,16 +2800,16 @@
         <v>18</v>
       </c>
       <c r="D39" t="s">
+        <v>157</v>
+      </c>
+      <c r="E39" t="s">
+        <v>20</v>
+      </c>
+      <c r="F39" t="s">
         <v>158</v>
       </c>
-      <c r="E39" t="s">
-        <v>20</v>
-      </c>
-      <c r="F39" t="s">
+      <c r="G39" t="s">
         <v>159</v>
-      </c>
-      <c r="G39" t="s">
-        <v>160</v>
       </c>
       <c r="H39" t="s">
         <v>22</v>
@@ -2833,7 +2833,7 @@
         <v>23</v>
       </c>
       <c r="R39" s="8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.25">
@@ -2844,16 +2844,16 @@
         <v>26</v>
       </c>
       <c r="D40" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E40" t="s">
         <v>20</v>
       </c>
       <c r="F40" t="s">
+        <v>165</v>
+      </c>
+      <c r="G40" t="s">
         <v>166</v>
-      </c>
-      <c r="G40" t="s">
-        <v>167</v>
       </c>
       <c r="H40" t="s">
         <v>22</v>
@@ -2878,7 +2878,7 @@
         <v>23</v>
       </c>
       <c r="R40" s="8" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>